<commit_message>
fix(): changement dans le tableau de synthèse.
</commit_message>
<xml_diff>
--- a/E5 - Tableau de synthèse.xlsx
+++ b/E5 - Tableau de synthèse.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp64\www\portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A06AE9B5-CAF0-40F7-91F0-C48EA37E7070}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D82B86D-63B9-43D5-B859-113262598117}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="12090" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E5" sheetId="1" r:id="rId1"/>
@@ -39,18 +39,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="50">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
   <si>
-    <t>SESSION 2025</t>
-  </si>
-  <si>
     <t xml:space="preserve">Tableau de synthèse des réalisations professionnelles </t>
-  </si>
-  <si>
-    <t xml:space="preserve">N° candidat : </t>
   </si>
   <si>
     <t>Option :</t>
@@ -123,15 +117,9 @@
     <t>Réalisations en milieu professionnel en cours de première année</t>
   </si>
   <si>
-    <t>Siteweb de gestion d'élévé pour un lycée (symfony,php)</t>
-  </si>
-  <si>
     <t>Réalisations en milieu professionnel en cours de seconde année</t>
   </si>
   <si>
-    <t>Mise à jour du site simple site.gouv (django , python , js )</t>
-  </si>
-  <si>
     <t xml:space="preserve">  </t>
   </si>
   <si>
@@ -156,9 +144,6 @@
     <t>Projet TO DO List fx (javaFX)</t>
   </si>
   <si>
-    <t>Adresse URL du portfolio : https://languithomas.wordpress.com</t>
-  </si>
-  <si>
     <t>SLAM</t>
   </si>
   <si>
@@ -196,6 +181,33 @@
   </si>
   <si>
     <t>X</t>
+  </si>
+  <si>
+    <t>Remplacement de Matériel Utilisateur</t>
+  </si>
+  <si>
+    <t>Remise de Matériel Utilisateur</t>
+  </si>
+  <si>
+    <t>Préparation de Poste pour le Télétravail</t>
+  </si>
+  <si>
+    <t>Gestion de ticketing</t>
+  </si>
+  <si>
+    <t>Mai - Juin</t>
+  </si>
+  <si>
+    <t>10/09/2025 - ...</t>
+  </si>
+  <si>
+    <t>Adresse URL du portfolio : https://tetard1.github.io/Portfolio/</t>
+  </si>
+  <si>
+    <t>N° candidat : 02247820814 - 003</t>
+  </si>
+  <si>
+    <t>SESSION 2025 - 2026</t>
   </si>
 </sst>
 </file>
@@ -740,9 +752,48 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -765,45 +816,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1125,122 +1137,122 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23" t="s">
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25" t="s">
+        <v>49</v>
+      </c>
+      <c r="H1" s="25"/>
+    </row>
+    <row r="2" spans="1:43" ht="41.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="23"/>
-    </row>
-    <row r="2" spans="1:43" ht="41.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="23" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
     </row>
     <row r="3" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="24" t="s">
-        <v>25</v>
-      </c>
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
-      <c r="E3" s="26"/>
-      <c r="F3" s="30" t="s">
-        <v>3</v>
-      </c>
-      <c r="G3" s="25"/>
-      <c r="H3" s="31"/>
+      <c r="A3" s="37" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="38"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="39"/>
+      <c r="F3" s="43" t="s">
+        <v>48</v>
+      </c>
+      <c r="G3" s="38"/>
+      <c r="H3" s="44"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="27" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" s="28"/>
-      <c r="C4" s="28"/>
-      <c r="D4" s="28"/>
-      <c r="E4" s="29"/>
+      <c r="A4" s="40" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="41"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="42"/>
       <c r="F4" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="G4" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" s="19"/>
+    </row>
+    <row r="5" spans="1:43" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="34" t="s">
+        <v>47</v>
+      </c>
+      <c r="B5" s="35"/>
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
+      <c r="E5" s="35"/>
+      <c r="F5" s="35"/>
+      <c r="G5" s="35"/>
+      <c r="H5" s="36"/>
+    </row>
+    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="G4" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="H4" s="19"/>
-    </row>
-    <row r="5" spans="1:43" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="42" t="s">
-        <v>32</v>
-      </c>
-      <c r="B5" s="43"/>
-      <c r="C5" s="43"/>
-      <c r="D5" s="43"/>
-      <c r="E5" s="43"/>
-      <c r="F5" s="43"/>
-      <c r="G5" s="43"/>
-      <c r="H5" s="44"/>
-    </row>
-    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="32" t="s">
+      <c r="C6" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="40" t="s">
+      <c r="D6" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="F6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="G6" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="H6" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="G6" s="6" t="s">
+    </row>
+    <row r="7" spans="1:43" s="2" customFormat="1" ht="325" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="24"/>
+      <c r="B7" s="33"/>
+      <c r="C7" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="D7" s="20" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="7" spans="1:43" s="2" customFormat="1" ht="325" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="33"/>
-      <c r="B7" s="41"/>
-      <c r="C7" s="20" t="s">
+      <c r="E7" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="F7" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="20" t="s">
+      <c r="G7" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="20" t="s">
+      <c r="H7" s="21" t="s">
         <v>16</v>
-      </c>
-      <c r="G7" s="20" t="s">
-        <v>17</v>
-      </c>
-      <c r="H7" s="21" t="s">
-        <v>18</v>
       </c>
       <c r="I7"/>
       <c r="J7"/>
@@ -1279,16 +1291,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A8" s="34" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" s="35"/>
-      <c r="C8" s="35"/>
-      <c r="D8" s="35"/>
-      <c r="E8" s="35"/>
-      <c r="F8" s="35"/>
-      <c r="G8" s="35"/>
-      <c r="H8" s="36"/>
+      <c r="A8" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="27"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="28"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1327,13 +1339,13 @@
     </row>
     <row r="9" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D9" s="22"/>
       <c r="E9" s="22"/>
@@ -1378,18 +1390,18 @@
     </row>
     <row r="10" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D10" s="15"/>
       <c r="E10" s="15"/>
       <c r="F10" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G10" s="15"/>
       <c r="H10" s="16"/>
@@ -1431,25 +1443,25 @@
     </row>
     <row r="11" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="H11" s="16"/>
       <c r="I11"/>
@@ -1490,25 +1502,25 @@
     </row>
     <row r="12" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="H12" s="16"/>
       <c r="I12"/>
@@ -1549,13 +1561,13 @@
     </row>
     <row r="13" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="8" t="s">
-        <v>36</v>
-      </c>
       <c r="C13" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D13" s="15"/>
       <c r="E13" s="15"/>
@@ -1600,28 +1612,28 @@
     </row>
     <row r="14" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="H14" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="I14"/>
       <c r="J14"/>
@@ -1661,25 +1673,25 @@
     </row>
     <row r="15" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F15" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G15" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="H15" s="16"/>
       <c r="I15"/>
@@ -1720,20 +1732,20 @@
     </row>
     <row r="16" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="E16" s="15"/>
       <c r="F16" s="14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G16" s="15"/>
       <c r="H16" s="16"/>
@@ -1864,16 +1876,16 @@
       <c r="AQ18"/>
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A19" s="37" t="s">
-        <v>20</v>
-      </c>
-      <c r="B19" s="38"/>
-      <c r="C19" s="38"/>
-      <c r="D19" s="38"/>
-      <c r="E19" s="38"/>
-      <c r="F19" s="38"/>
-      <c r="G19" s="38"/>
-      <c r="H19" s="39"/>
+      <c r="A19" s="29" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="30"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="30"/>
+      <c r="G19" s="30"/>
+      <c r="H19" s="31"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1912,14 +1924,20 @@
     </row>
     <row r="20" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B20" s="8"/>
+        <v>41</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>45</v>
+      </c>
       <c r="C20" s="15"/>
-      <c r="D20" s="15"/>
+      <c r="D20" s="14" t="s">
+        <v>40</v>
+      </c>
       <c r="E20" s="15"/>
       <c r="F20" s="15"/>
-      <c r="G20" s="15"/>
+      <c r="G20" s="14" t="s">
+        <v>40</v>
+      </c>
       <c r="H20" s="16"/>
       <c r="I20"/>
       <c r="J20"/>
@@ -1958,13 +1976,21 @@
       <c r="AQ20"/>
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="9"/>
-      <c r="B21" s="8"/>
+      <c r="A21" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>45</v>
+      </c>
       <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
+      <c r="D21" s="14" t="s">
+        <v>40</v>
+      </c>
       <c r="E21" s="15"/>
       <c r="F21" s="15"/>
-      <c r="G21" s="15"/>
+      <c r="G21" s="14" t="s">
+        <v>40</v>
+      </c>
       <c r="H21" s="16"/>
       <c r="I21"/>
       <c r="J21"/>
@@ -2003,13 +2029,21 @@
       <c r="AQ21"/>
     </row>
     <row r="22" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="9"/>
-      <c r="B22" s="8"/>
+      <c r="A22" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>45</v>
+      </c>
       <c r="C22" s="15"/>
-      <c r="D22" s="15"/>
+      <c r="D22" s="14" t="s">
+        <v>40</v>
+      </c>
       <c r="E22" s="15"/>
       <c r="F22" s="15"/>
-      <c r="G22" s="15"/>
+      <c r="G22" s="14" t="s">
+        <v>40</v>
+      </c>
       <c r="H22" s="16"/>
       <c r="I22"/>
       <c r="J22"/>
@@ -2048,13 +2082,21 @@
       <c r="AQ22"/>
     </row>
     <row r="23" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="9"/>
-      <c r="B23" s="8"/>
+      <c r="A23" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>45</v>
+      </c>
       <c r="C23" s="15"/>
-      <c r="D23" s="15"/>
+      <c r="D23" s="14" t="s">
+        <v>40</v>
+      </c>
       <c r="E23" s="15"/>
       <c r="F23" s="15"/>
-      <c r="G23" s="15"/>
+      <c r="G23" s="14" t="s">
+        <v>40</v>
+      </c>
       <c r="H23" s="16"/>
       <c r="I23"/>
       <c r="J23"/>
@@ -2228,16 +2270,16 @@
       <c r="AQ26"/>
     </row>
     <row r="27" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A27" s="37" t="s">
-        <v>22</v>
-      </c>
-      <c r="B27" s="38"/>
-      <c r="C27" s="38"/>
-      <c r="D27" s="38"/>
-      <c r="E27" s="38"/>
-      <c r="F27" s="38"/>
-      <c r="G27" s="38"/>
-      <c r="H27" s="39"/>
+      <c r="A27" s="29" t="s">
+        <v>19</v>
+      </c>
+      <c r="B27" s="30"/>
+      <c r="C27" s="30"/>
+      <c r="D27" s="30"/>
+      <c r="E27" s="30"/>
+      <c r="F27" s="30"/>
+      <c r="G27" s="30"/>
+      <c r="H27" s="31"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2276,14 +2318,20 @@
     </row>
     <row r="28" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B28" s="8"/>
+        <v>41</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>46</v>
+      </c>
       <c r="C28" s="15"/>
-      <c r="D28" s="15"/>
+      <c r="D28" s="14" t="s">
+        <v>40</v>
+      </c>
       <c r="E28" s="15"/>
       <c r="F28" s="15"/>
-      <c r="G28" s="15"/>
+      <c r="G28" s="14" t="s">
+        <v>40</v>
+      </c>
       <c r="H28" s="16"/>
       <c r="I28"/>
       <c r="J28"/>
@@ -2322,13 +2370,21 @@
       <c r="AQ28"/>
     </row>
     <row r="29" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="9"/>
-      <c r="B29" s="8"/>
+      <c r="A29" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>46</v>
+      </c>
       <c r="C29" s="15"/>
-      <c r="D29" s="15"/>
+      <c r="D29" s="14" t="s">
+        <v>40</v>
+      </c>
       <c r="E29" s="15"/>
       <c r="F29" s="15"/>
-      <c r="G29" s="15"/>
+      <c r="G29" s="14" t="s">
+        <v>40</v>
+      </c>
       <c r="H29" s="16"/>
       <c r="I29"/>
       <c r="J29"/>
@@ -2367,13 +2423,21 @@
       <c r="AQ29"/>
     </row>
     <row r="30" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="9"/>
-      <c r="B30" s="8"/>
+      <c r="A30" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>46</v>
+      </c>
       <c r="C30" s="15"/>
-      <c r="D30" s="15"/>
+      <c r="D30" s="14" t="s">
+        <v>40</v>
+      </c>
       <c r="E30" s="15"/>
       <c r="F30" s="15"/>
-      <c r="G30" s="15"/>
+      <c r="G30" s="14" t="s">
+        <v>40</v>
+      </c>
       <c r="H30" s="16"/>
       <c r="I30"/>
       <c r="J30"/>
@@ -2387,7 +2451,7 @@
       <c r="R30"/>
       <c r="S30"/>
       <c r="T30" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="U30"/>
       <c r="V30"/>
@@ -2414,13 +2478,21 @@
       <c r="AQ30"/>
     </row>
     <row r="31" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="9"/>
-      <c r="B31" s="8"/>
+      <c r="A31" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>46</v>
+      </c>
       <c r="C31" s="15"/>
-      <c r="D31" s="15"/>
+      <c r="D31" s="14" t="s">
+        <v>40</v>
+      </c>
       <c r="E31" s="15"/>
       <c r="F31" s="15"/>
-      <c r="G31" s="15"/>
+      <c r="G31" s="14" t="s">
+        <v>40</v>
+      </c>
       <c r="H31" s="16"/>
       <c r="I31"/>
       <c r="J31"/>
@@ -2686,6 +2758,11 @@
     <row r="81" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2693,11 +2770,6 @@
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -2708,26 +2780,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a81de258-2782-43d6-9d1d-cd28d60619af">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ed3c7b2c-ee95-4c62-b749-48a072e0fc6f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009F94F24C812C1443AF756F3262092C76" ma:contentTypeVersion="12" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="151ba19e32653bee0a5eee1707588175">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a81de258-2782-43d6-9d1d-cd28d60619af" xmlns:ns3="ed3c7b2c-ee95-4c62-b749-48a072e0fc6f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="177f0ace5463b349477f87f1b4642be3" ns2:_="" ns3:_="">
     <xsd:import namespace="a81de258-2782-43d6-9d1d-cd28d60619af"/>
@@ -2928,10 +2980,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a81de258-2782-43d6-9d1d-cd28d60619af">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ed3c7b2c-ee95-4c62-b749-48a072e0fc6f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AE36CC0-C123-4309-B645-BEFA7CB5FE5A}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4E8AC1FA-2BD8-42E8-B266-319DE6BBF638}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="a81de258-2782-43d6-9d1d-cd28d60619af"/>
+    <ds:schemaRef ds:uri="ed3c7b2c-ee95-4c62-b749-48a072e0fc6f"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2948,20 +3031,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4E8AC1FA-2BD8-42E8-B266-319DE6BBF638}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AE36CC0-C123-4309-B645-BEFA7CB5FE5A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="a81de258-2782-43d6-9d1d-cd28d60619af"/>
-    <ds:schemaRef ds:uri="ed3c7b2c-ee95-4c62-b749-48a072e0fc6f"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fix(): modification dans le tableau de synthèse.
</commit_message>
<xml_diff>
--- a/E5 - Tableau de synthèse.xlsx
+++ b/E5 - Tableau de synthèse.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp64\www\portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D82B86D-63B9-43D5-B859-113262598117}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0CD48F2-D0B4-42D4-A1A8-7F261A0D52BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="50">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -752,15 +752,39 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -792,30 +816,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1137,56 +1137,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25" t="s">
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="H1" s="25"/>
+      <c r="H1" s="23"/>
     </row>
     <row r="2" spans="1:43" ht="41.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
     </row>
     <row r="3" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="37" t="s">
+      <c r="A3" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="38"/>
-      <c r="C3" s="38"/>
-      <c r="D3" s="38"/>
-      <c r="E3" s="39"/>
-      <c r="F3" s="43" t="s">
+      <c r="B3" s="25"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="30" t="s">
         <v>48</v>
       </c>
-      <c r="G3" s="38"/>
-      <c r="H3" s="44"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="31"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="40" t="s">
+      <c r="A4" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="41"/>
-      <c r="C4" s="41"/>
-      <c r="D4" s="41"/>
-      <c r="E4" s="42"/>
+      <c r="B4" s="28"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="29"/>
       <c r="F4" s="12" t="s">
         <v>2</v>
       </c>
@@ -1196,22 +1196,22 @@
       <c r="H4" s="19"/>
     </row>
     <row r="5" spans="1:43" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="34" t="s">
+      <c r="A5" s="42" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="35"/>
-      <c r="C5" s="35"/>
-      <c r="D5" s="35"/>
-      <c r="E5" s="35"/>
-      <c r="F5" s="35"/>
-      <c r="G5" s="35"/>
-      <c r="H5" s="36"/>
+      <c r="B5" s="43"/>
+      <c r="C5" s="43"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="44"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="23" t="s">
+      <c r="A6" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="B6" s="40" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1234,8 +1234,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="325" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="24"/>
-      <c r="B7" s="33"/>
+      <c r="A7" s="33"/>
+      <c r="B7" s="41"/>
       <c r="C7" s="20" t="s">
         <v>11</v>
       </c>
@@ -1291,16 +1291,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A8" s="26" t="s">
+      <c r="A8" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="27"/>
-      <c r="C8" s="27"/>
-      <c r="D8" s="27"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="28"/>
+      <c r="B8" s="35"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="35"/>
+      <c r="E8" s="35"/>
+      <c r="F8" s="35"/>
+      <c r="G8" s="35"/>
+      <c r="H8" s="36"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1876,16 +1876,16 @@
       <c r="AQ18"/>
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A19" s="29" t="s">
+      <c r="A19" s="37" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="30"/>
-      <c r="C19" s="30"/>
-      <c r="D19" s="30"/>
-      <c r="E19" s="30"/>
-      <c r="F19" s="30"/>
-      <c r="G19" s="30"/>
-      <c r="H19" s="31"/>
+      <c r="B19" s="38"/>
+      <c r="C19" s="38"/>
+      <c r="D19" s="38"/>
+      <c r="E19" s="38"/>
+      <c r="F19" s="38"/>
+      <c r="G19" s="38"/>
+      <c r="H19" s="39"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1929,7 +1929,9 @@
       <c r="B20" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="15"/>
+      <c r="C20" s="14" t="s">
+        <v>40</v>
+      </c>
       <c r="D20" s="14" t="s">
         <v>40</v>
       </c>
@@ -1982,7 +1984,9 @@
       <c r="B21" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="C21" s="15"/>
+      <c r="C21" s="14" t="s">
+        <v>40</v>
+      </c>
       <c r="D21" s="14" t="s">
         <v>40</v>
       </c>
@@ -2035,7 +2039,9 @@
       <c r="B22" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="C22" s="15"/>
+      <c r="C22" s="14" t="s">
+        <v>40</v>
+      </c>
       <c r="D22" s="14" t="s">
         <v>40</v>
       </c>
@@ -2088,7 +2094,9 @@
       <c r="B23" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="C23" s="15"/>
+      <c r="C23" s="14" t="s">
+        <v>40</v>
+      </c>
       <c r="D23" s="14" t="s">
         <v>40</v>
       </c>
@@ -2270,16 +2278,16 @@
       <c r="AQ26"/>
     </row>
     <row r="27" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A27" s="29" t="s">
+      <c r="A27" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="B27" s="30"/>
-      <c r="C27" s="30"/>
-      <c r="D27" s="30"/>
-      <c r="E27" s="30"/>
-      <c r="F27" s="30"/>
-      <c r="G27" s="30"/>
-      <c r="H27" s="31"/>
+      <c r="B27" s="38"/>
+      <c r="C27" s="38"/>
+      <c r="D27" s="38"/>
+      <c r="E27" s="38"/>
+      <c r="F27" s="38"/>
+      <c r="G27" s="38"/>
+      <c r="H27" s="39"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2323,7 +2331,9 @@
       <c r="B28" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C28" s="15"/>
+      <c r="C28" s="14" t="s">
+        <v>40</v>
+      </c>
       <c r="D28" s="14" t="s">
         <v>40</v>
       </c>
@@ -2376,7 +2386,9 @@
       <c r="B29" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C29" s="15"/>
+      <c r="C29" s="14" t="s">
+        <v>40</v>
+      </c>
       <c r="D29" s="14" t="s">
         <v>40</v>
       </c>
@@ -2429,7 +2441,9 @@
       <c r="B30" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C30" s="15"/>
+      <c r="C30" s="14" t="s">
+        <v>40</v>
+      </c>
       <c r="D30" s="14" t="s">
         <v>40</v>
       </c>
@@ -2484,7 +2498,9 @@
       <c r="B31" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C31" s="15"/>
+      <c r="C31" s="14" t="s">
+        <v>40</v>
+      </c>
       <c r="D31" s="14" t="s">
         <v>40</v>
       </c>
@@ -2758,11 +2774,6 @@
     <row r="81" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2770,6 +2781,11 @@
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -2780,6 +2796,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a81de258-2782-43d6-9d1d-cd28d60619af">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ed3c7b2c-ee95-4c62-b749-48a072e0fc6f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009F94F24C812C1443AF756F3262092C76" ma:contentTypeVersion="12" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="151ba19e32653bee0a5eee1707588175">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a81de258-2782-43d6-9d1d-cd28d60619af" xmlns:ns3="ed3c7b2c-ee95-4c62-b749-48a072e0fc6f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="177f0ace5463b349477f87f1b4642be3" ns2:_="" ns3:_="">
     <xsd:import namespace="a81de258-2782-43d6-9d1d-cd28d60619af"/>
@@ -2980,27 +3016,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a81de258-2782-43d6-9d1d-cd28d60619af">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ed3c7b2c-ee95-4c62-b749-48a072e0fc6f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AE36CC0-C123-4309-B645-BEFA7CB5FE5A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76E9F743-2553-4538-B86E-9E9E949B7313}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a81de258-2782-43d6-9d1d-cd28d60619af"/>
+    <ds:schemaRef ds:uri="ed3c7b2c-ee95-4c62-b749-48a072e0fc6f"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4E8AC1FA-2BD8-42E8-B266-319DE6BBF638}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3017,23 +3052,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76E9F743-2553-4538-B86E-9E9E949B7313}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a81de258-2782-43d6-9d1d-cd28d60619af"/>
-    <ds:schemaRef ds:uri="ed3c7b2c-ee95-4c62-b749-48a072e0fc6f"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AE36CC0-C123-4309-B645-BEFA7CB5FE5A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>